<commit_message>
Added some remarks on my latest scalability issue with the code.
</commit_message>
<xml_diff>
--- a/high-level/assessment.xlsx
+++ b/high-level/assessment.xlsx
@@ -5,12 +5,13 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Coversheet" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Core" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Intra-node" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Labelling" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -22,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="61">
   <si>
     <t xml:space="preserve">High-level Performance Assessment</t>
   </si>
@@ -148,15 +149,74 @@
   </si>
   <si>
     <t xml:space="preserve">E (Amdahl)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Labelling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Function</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Effective Time (percentage)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Does Science</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Effective Science</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Overhead</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tarch::la::invert&lt;(int)36, double&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tarch::la::lu&lt;(int)36, double&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tarch::la::matVec&lt;(int)96, (int)36, double&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">peano4::grid::GridTraversalEventGenerator::getVertexType</t>
+  </si>
+  <si>
+    <t xml:space="preserve">__intel_avx_rep_memcpy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">peano4::parallel::Node::getLocalTreeId</t>
+  </si>
+  <si>
+    <t xml:space="preserve">__intel_avx_rep_memset</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tarch::la::matVec&lt;(int)36, (int)48, double&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tarch::la::Matrix&lt;(int)36, (int)36, double&gt;::operator()</t>
+  </si>
+  <si>
+    <t xml:space="preserve">peano4::datamanagement::CellMarker::CellMarker</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Top-10 time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiny routines</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Summary</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="General"/>
+    <numFmt numFmtId="166" formatCode="0.00%"/>
+    <numFmt numFmtId="167" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -283,7 +343,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="21">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -324,15 +384,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -352,7 +404,27 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -520,11 +592,16 @@
               <a:p>
                 <a:pPr>
                   <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:latin typeface="Arial"/>
+                    <a:ea typeface="DejaVu Sans"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="r"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
@@ -622,11 +699,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="36312737"/>
-        <c:axId val="6823514"/>
+        <c:axId val="11288364"/>
+        <c:axId val="24949475"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="36312737"/>
+        <c:axId val="11288364"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -658,7 +735,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="6823514"/>
+        <c:crossAx val="24949475"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -666,7 +743,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="6823514"/>
+        <c:axId val="24949475"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -707,7 +784,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="36312737"/>
+        <c:crossAx val="11288364"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -780,9 +857,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>504720</xdr:colOff>
+      <xdr:colOff>504360</xdr:colOff>
       <xdr:row>9</xdr:row>
-      <xdr:rowOff>27720</xdr:rowOff>
+      <xdr:rowOff>27360</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -796,7 +873,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="412920"/>
-          <a:ext cx="1553760" cy="1165320"/>
+          <a:ext cx="1553400" cy="1164960"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -817,9 +894,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>4238280</xdr:colOff>
+      <xdr:colOff>4237920</xdr:colOff>
       <xdr:row>8</xdr:row>
-      <xdr:rowOff>141840</xdr:rowOff>
+      <xdr:rowOff>141480</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -833,7 +910,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1901160" y="532440"/>
-          <a:ext cx="3386160" cy="997560"/>
+          <a:ext cx="3385800" cy="997200"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -859,9 +936,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>1553760</xdr:colOff>
+      <xdr:colOff>1553400</xdr:colOff>
       <xdr:row>9</xdr:row>
-      <xdr:rowOff>27720</xdr:rowOff>
+      <xdr:rowOff>27360</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -875,7 +952,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="412920"/>
-          <a:ext cx="1553760" cy="1165320"/>
+          <a:ext cx="1553400" cy="1164960"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -896,9 +973,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>680400</xdr:colOff>
+      <xdr:colOff>680040</xdr:colOff>
       <xdr:row>8</xdr:row>
-      <xdr:rowOff>113040</xdr:rowOff>
+      <xdr:rowOff>112680</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -912,7 +989,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1911960" y="503640"/>
-          <a:ext cx="3386160" cy="997560"/>
+          <a:ext cx="3385080" cy="997200"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -938,9 +1015,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>504720</xdr:colOff>
+      <xdr:colOff>504360</xdr:colOff>
       <xdr:row>9</xdr:row>
-      <xdr:rowOff>27720</xdr:rowOff>
+      <xdr:rowOff>27360</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -954,7 +1031,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="412920"/>
-          <a:ext cx="1553760" cy="1165320"/>
+          <a:ext cx="1553400" cy="1164960"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -975,9 +1052,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>4238280</xdr:colOff>
+      <xdr:colOff>4237920</xdr:colOff>
       <xdr:row>8</xdr:row>
-      <xdr:rowOff>141840</xdr:rowOff>
+      <xdr:rowOff>141480</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -991,7 +1068,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1901160" y="532440"/>
-          <a:ext cx="3386160" cy="997560"/>
+          <a:ext cx="3385800" cy="997200"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1012,9 +1089,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>575640</xdr:colOff>
+      <xdr:colOff>575280</xdr:colOff>
       <xdr:row>34</xdr:row>
-      <xdr:rowOff>37440</xdr:rowOff>
+      <xdr:rowOff>37080</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1023,7 +1100,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="7577640" y="6040440"/>
-        <a:ext cx="5758920" cy="3238920"/>
+        <a:ext cx="5758560" cy="3238560"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -1031,6 +1108,85 @@
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>740520</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>27360</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Image 7" descr=""/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="412920"/>
+          <a:ext cx="1553400" cy="1164960"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>107280</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>119520</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>3493080</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>141480</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Image 8" descr=""/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="920160" y="532440"/>
+          <a:ext cx="3385800" cy="997200"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -1242,7 +1398,7 @@
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="44.65"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="20.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="20.85"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="57.17"/>
   </cols>
   <sheetData>
@@ -1353,7 +1509,6 @@
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4"/>
       <c r="B23" s="9"/>
-      <c r="C23" s="0"/>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
@@ -1384,11 +1539,8 @@
         <v>20</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="0"/>
-    </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="10" t="s">
+      <c r="A28" s="7" t="s">
         <v>28</v>
       </c>
     </row>
@@ -1396,7 +1548,7 @@
       <c r="A29" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B29" s="11" t="n">
+      <c r="B29" s="10" t="n">
         <f aca="false">B21/B25</f>
         <v>0.397311715650674</v>
       </c>
@@ -1405,7 +1557,7 @@
       <c r="A30" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B30" s="11" t="n">
+      <c r="B30" s="10" t="n">
         <f aca="false">B22/B26</f>
         <v>0.224841571235796</v>
       </c>
@@ -1414,7 +1566,7 @@
       <c r="A32" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B32" s="12"/>
+      <c r="B32" s="9"/>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="5"/>
@@ -1496,13 +1648,13 @@
       <c r="A15" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="B15" s="13" t="s">
+      <c r="B15" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="C15" s="14" t="s">
+      <c r="C15" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="D15" s="14" t="s">
+      <c r="D15" s="12" t="s">
         <v>37</v>
       </c>
       <c r="E15" s="7" t="s">
@@ -1519,7 +1671,7 @@
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="15" t="n">
+      <c r="A16" s="13" t="n">
         <v>1</v>
       </c>
       <c r="B16" s="5" t="n">
@@ -1533,24 +1685,24 @@
         <f aca="false">$B$16/B16</f>
         <v>1</v>
       </c>
-      <c r="E16" s="11" t="n">
+      <c r="E16" s="10" t="n">
         <f aca="false">$B$14/$B$16</f>
         <v>0.956628839967953</v>
       </c>
-      <c r="F16" s="0" t="n">
+      <c r="F16" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="G16" s="11" t="n">
+      <c r="G16" s="10" t="n">
         <f aca="false">C16/A16</f>
         <v>0.956628839967953</v>
       </c>
-      <c r="H16" s="11" t="n">
+      <c r="H16" s="10" t="n">
         <f aca="false">D16/A16</f>
         <v>1</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="16.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="16" t="n">
+      <c r="A17" s="14" t="n">
         <v>2</v>
       </c>
       <c r="B17" s="5" t="n">
@@ -1564,25 +1716,25 @@
         <f aca="false">$B$16/B17</f>
         <v>1.71464833378099</v>
       </c>
-      <c r="E17" s="11" t="n">
+      <c r="E17" s="10" t="n">
         <f aca="false">$B$14/$B$16</f>
         <v>0.956628839967953</v>
       </c>
-      <c r="F17" s="17" t="n">
+      <c r="F17" s="1" t="n">
         <f aca="false">(B17/B$16-1)/(1/A17-1)</f>
         <v>0.833580063854975</v>
       </c>
-      <c r="G17" s="11" t="n">
+      <c r="G17" s="10" t="n">
         <f aca="false">C17/A17</f>
-        <v>0.82014102324895</v>
-      </c>
-      <c r="H17" s="11" t="n">
+        <v>0.820141023248948</v>
+      </c>
+      <c r="H17" s="10" t="n">
         <f aca="false">D17/A17</f>
         <v>0.857324166890497</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="16" t="n">
+      <c r="A18" s="14" t="n">
         <v>3</v>
       </c>
       <c r="B18" s="5" t="n">
@@ -1596,25 +1748,25 @@
         <f aca="false">$B$16/B18</f>
         <v>2.29336865516513</v>
       </c>
-      <c r="E18" s="11" t="n">
+      <c r="E18" s="10" t="n">
         <f aca="false">$B$14/$B$16</f>
         <v>0.956628839967953</v>
       </c>
-      <c r="F18" s="17" t="n">
+      <c r="F18" s="1" t="n">
         <f aca="false">(B18/B$16-1)/(1/A18-1)</f>
         <v>0.845940306360386</v>
       </c>
-      <c r="G18" s="11" t="n">
+      <c r="G18" s="10" t="n">
         <f aca="false">C18/A18</f>
-        <v>0.731300865403163</v>
-      </c>
-      <c r="H18" s="11" t="n">
+        <v>0.731300865403162</v>
+      </c>
+      <c r="H18" s="10" t="n">
         <f aca="false">D18/A18</f>
         <v>0.764456218388378</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="16" t="n">
+      <c r="A19" s="14" t="n">
         <v>4</v>
       </c>
       <c r="B19" s="5" t="n">
@@ -1628,25 +1780,25 @@
         <f aca="false">$B$16/B19</f>
         <v>2.88546073106942</v>
       </c>
-      <c r="E19" s="11" t="n">
+      <c r="E19" s="10" t="n">
         <f aca="false">$B$14/$B$16</f>
         <v>0.956628839967953</v>
       </c>
-      <c r="F19" s="17" t="n">
+      <c r="F19" s="1" t="n">
         <f aca="false">(B19/B$16-1)/(1/A19-1)</f>
         <v>0.871246527238013</v>
       </c>
-      <c r="G19" s="11" t="n">
+      <c r="G19" s="10" t="n">
         <f aca="false">C19/A19</f>
-        <v>0.690078737984005</v>
-      </c>
-      <c r="H19" s="11" t="n">
+        <v>0.690078737984004</v>
+      </c>
+      <c r="H19" s="10" t="n">
         <f aca="false">D19/A19</f>
         <v>0.721365182767354</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="15" t="n">
+      <c r="A20" s="13" t="n">
         <v>6</v>
       </c>
       <c r="B20" s="5" t="n">
@@ -1660,25 +1812,25 @@
         <f aca="false">$B$16/B20</f>
         <v>4.10757790089984</v>
       </c>
-      <c r="E20" s="11" t="n">
+      <c r="E20" s="10" t="n">
         <f aca="false">$B$14/$B$16</f>
         <v>0.956628839967953</v>
       </c>
-      <c r="F20" s="17" t="n">
+      <c r="F20" s="1" t="n">
         <f aca="false">(B20/B$16-1)/(1/A20-1)</f>
         <v>0.907857031819867</v>
       </c>
-      <c r="G20" s="11" t="n">
+      <c r="G20" s="10" t="n">
         <f aca="false">C20/A20</f>
         <v>0.654904580402635</v>
       </c>
-      <c r="H20" s="11" t="n">
+      <c r="H20" s="10" t="n">
         <f aca="false">D20/A20</f>
         <v>0.68459631681664</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="15" t="n">
+      <c r="A21" s="13" t="n">
         <v>8</v>
       </c>
       <c r="B21" s="5" t="n">
@@ -1692,25 +1844,25 @@
         <f aca="false">$B$16/B21</f>
         <v>4.85021952337039</v>
       </c>
-      <c r="E21" s="11" t="n">
+      <c r="E21" s="10" t="n">
         <f aca="false">$B$14/$B$16</f>
         <v>0.956628839967953</v>
       </c>
-      <c r="F21" s="17" t="n">
+      <c r="F21" s="1" t="n">
         <f aca="false">(B21/B$16-1)/(1/A21-1)</f>
         <v>0.907227160059379</v>
       </c>
-      <c r="G21" s="11" t="n">
+      <c r="G21" s="10" t="n">
         <f aca="false">C21/A21</f>
         <v>0.579982484528967</v>
       </c>
-      <c r="H21" s="11" t="n">
+      <c r="H21" s="10" t="n">
         <f aca="false">D21/A21</f>
         <v>0.606277440421299</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="15" t="n">
+      <c r="A22" s="13" t="n">
         <v>10</v>
       </c>
       <c r="B22" s="5"/>
@@ -1722,25 +1874,25 @@
         <f aca="false">$B$16/B22</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E22" s="11" t="n">
+      <c r="E22" s="10" t="n">
         <f aca="false">$B$14/$B$16</f>
         <v>0.956628839967953</v>
       </c>
-      <c r="F22" s="17" t="n">
+      <c r="F22" s="1" t="n">
         <f aca="false">(B22/B$16-1)/(1/A22-1)</f>
         <v>1.11111111111111</v>
       </c>
-      <c r="G22" s="11" t="e">
+      <c r="G22" s="10" t="e">
         <f aca="false">C22/A22</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="H22" s="11" t="e">
+      <c r="H22" s="10" t="e">
         <f aca="false">D22/A22</f>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="15" t="n">
+      <c r="A23" s="13" t="n">
         <v>12</v>
       </c>
       <c r="B23" s="5"/>
@@ -1752,25 +1904,25 @@
         <f aca="false">$B$16/B23</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E23" s="11" t="n">
+      <c r="E23" s="10" t="n">
         <f aca="false">$B$14/$B$16</f>
         <v>0.956628839967953</v>
       </c>
-      <c r="F23" s="17" t="n">
+      <c r="F23" s="1" t="n">
         <f aca="false">(B23/B$16-1)/(1/A23-1)</f>
         <v>1.09090909090909</v>
       </c>
-      <c r="G23" s="11" t="e">
+      <c r="G23" s="10" t="e">
         <f aca="false">C23/A23</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="H23" s="11" t="e">
+      <c r="H23" s="10" t="e">
         <f aca="false">D23/A23</f>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="15" t="n">
+      <c r="A24" s="13" t="n">
         <v>14</v>
       </c>
       <c r="B24" s="5"/>
@@ -1782,25 +1934,25 @@
         <f aca="false">$B$16/B24</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E24" s="11" t="n">
+      <c r="E24" s="10" t="n">
         <f aca="false">$B$14/$B$16</f>
         <v>0.956628839967953</v>
       </c>
-      <c r="F24" s="17" t="n">
+      <c r="F24" s="1" t="n">
         <f aca="false">(B24/B$16-1)/(1/A24-1)</f>
         <v>1.07692307692308</v>
       </c>
-      <c r="G24" s="11" t="e">
+      <c r="G24" s="10" t="e">
         <f aca="false">C24/A24</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="H24" s="11" t="e">
+      <c r="H24" s="10" t="e">
         <f aca="false">D24/A24</f>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="15" t="n">
+      <c r="A25" s="13" t="n">
         <v>16</v>
       </c>
       <c r="B25" s="5"/>
@@ -1812,25 +1964,25 @@
         <f aca="false">$B$16/B25</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E25" s="11" t="n">
+      <c r="E25" s="10" t="n">
         <f aca="false">$B$14/$B$16</f>
         <v>0.956628839967953</v>
       </c>
-      <c r="F25" s="17" t="n">
+      <c r="F25" s="1" t="n">
         <f aca="false">(B25/B$16-1)/(1/A25-1)</f>
         <v>1.06666666666667</v>
       </c>
-      <c r="G25" s="11" t="e">
+      <c r="G25" s="10" t="e">
         <f aca="false">C25/A25</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="H25" s="11" t="e">
+      <c r="H25" s="10" t="e">
         <f aca="false">D25/A25</f>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="15" t="n">
+      <c r="A26" s="13" t="n">
         <v>20</v>
       </c>
       <c r="B26" s="5"/>
@@ -1842,25 +1994,25 @@
         <f aca="false">$B$16/B26</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E26" s="11" t="n">
+      <c r="E26" s="10" t="n">
         <f aca="false">$B$14/$B$16</f>
         <v>0.956628839967953</v>
       </c>
-      <c r="F26" s="17" t="n">
+      <c r="F26" s="1" t="n">
         <f aca="false">(B26/B$16-1)/(1/A26-1)</f>
         <v>1.05263157894737</v>
       </c>
-      <c r="G26" s="11" t="e">
+      <c r="G26" s="10" t="e">
         <f aca="false">C26/A26</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="H26" s="11" t="e">
+      <c r="H26" s="10" t="e">
         <f aca="false">D26/A26</f>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="15" t="n">
+      <c r="A27" s="13" t="n">
         <v>24</v>
       </c>
       <c r="B27" s="5"/>
@@ -1872,25 +2024,25 @@
         <f aca="false">$B$16/B27</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E27" s="11" t="n">
+      <c r="E27" s="10" t="n">
         <f aca="false">$B$14/$B$16</f>
         <v>0.956628839967953</v>
       </c>
-      <c r="F27" s="17" t="n">
+      <c r="F27" s="1" t="n">
         <f aca="false">(B27/B$16-1)/(1/A27-1)</f>
         <v>1.04347826086957</v>
       </c>
-      <c r="G27" s="11" t="e">
+      <c r="G27" s="10" t="e">
         <f aca="false">C27/A27</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="H27" s="11" t="e">
+      <c r="H27" s="10" t="e">
         <f aca="false">D27/A27</f>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="15" t="n">
+      <c r="A28" s="13" t="n">
         <v>28</v>
       </c>
       <c r="B28" s="5"/>
@@ -1902,19 +2054,19 @@
         <f aca="false">$B$16/B28</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E28" s="11" t="n">
+      <c r="E28" s="10" t="n">
         <f aca="false">$B$14/$B$16</f>
         <v>0.956628839967953</v>
       </c>
-      <c r="F28" s="17" t="n">
+      <c r="F28" s="1" t="n">
         <f aca="false">(B28/B$16-1)/(1/A28-1)</f>
         <v>1.03703703703704</v>
       </c>
-      <c r="G28" s="11" t="e">
+      <c r="G28" s="10" t="e">
         <f aca="false">C28/A28</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="H28" s="11" t="e">
+      <c r="H28" s="10" t="e">
         <f aca="false">D28/A28</f>
         <v>#DIV/0!</v>
       </c>
@@ -1952,4 +2104,395 @@
   </headerFooter>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:G44"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="61.21"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1"/>
+      <c r="B7" s="1"/>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1"/>
+      <c r="B8" s="1"/>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1"/>
+      <c r="B9" s="1"/>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1"/>
+      <c r="B10" s="1"/>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1"/>
+    </row>
+    <row r="11" customFormat="false" ht="82.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1"/>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="C13" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="D13" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="E13" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="F13" s="15" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="C14" s="17" t="n">
+        <v>0.439</v>
+      </c>
+      <c r="D14" s="18" t="b">
+        <v>1</v>
+      </c>
+      <c r="E14" s="19" t="n">
+        <f aca="false">IF(D14,C14,0)</f>
+        <v>0.439</v>
+      </c>
+      <c r="F14" s="19" t="n">
+        <f aca="false">IF(E14,0,C14)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="C15" s="17" t="n">
+        <v>0.078</v>
+      </c>
+      <c r="D15" s="18" t="b">
+        <v>1</v>
+      </c>
+      <c r="E15" s="19" t="n">
+        <f aca="false">IF(D15,C15,0)</f>
+        <v>0.078</v>
+      </c>
+      <c r="F15" s="19" t="n">
+        <f aca="false">IF(E15,0,C15)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="C16" s="17" t="n">
+        <v>0.026</v>
+      </c>
+      <c r="D16" s="18" t="b">
+        <v>1</v>
+      </c>
+      <c r="E16" s="19" t="n">
+        <f aca="false">IF(D16,C16,0)</f>
+        <v>0.026</v>
+      </c>
+      <c r="F16" s="19" t="n">
+        <f aca="false">IF(E16,0,C16)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="C17" s="17" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="D17" s="18" t="b">
+        <v>0</v>
+      </c>
+      <c r="E17" s="19" t="n">
+        <f aca="false">IF(D17,C17,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F17" s="19" t="n">
+        <f aca="false">IF(E17,0,C17)</f>
+        <v>0.023</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="C18" s="17" t="n">
+        <v>0.017</v>
+      </c>
+      <c r="D18" s="18" t="b">
+        <v>0</v>
+      </c>
+      <c r="E18" s="19" t="n">
+        <f aca="false">IF(D18,C18,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F18" s="19" t="n">
+        <f aca="false">IF(E18,0,C18)</f>
+        <v>0.017</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="C19" s="17" t="n">
+        <v>0.016</v>
+      </c>
+      <c r="D19" s="18" t="b">
+        <v>0</v>
+      </c>
+      <c r="E19" s="19" t="n">
+        <f aca="false">IF(D19,C19,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F19" s="19" t="n">
+        <f aca="false">IF(E19,0,C19)</f>
+        <v>0.016</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="C20" s="17" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="D20" s="18" t="b">
+        <v>0</v>
+      </c>
+      <c r="E20" s="19" t="n">
+        <f aca="false">IF(D20,C20,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F20" s="19" t="n">
+        <f aca="false">IF(E20,0,C20)</f>
+        <v>0.013</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B21" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="C21" s="17" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="D21" s="18" t="b">
+        <v>1</v>
+      </c>
+      <c r="E21" s="19" t="n">
+        <f aca="false">IF(D21,C21,0)</f>
+        <v>0.013</v>
+      </c>
+      <c r="F21" s="19" t="n">
+        <f aca="false">IF(E21,0,C21)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="C22" s="17" t="n">
+        <v>0.009</v>
+      </c>
+      <c r="D22" s="18" t="b">
+        <v>1</v>
+      </c>
+      <c r="E22" s="19" t="n">
+        <f aca="false">IF(D22,C22,0)</f>
+        <v>0.009</v>
+      </c>
+      <c r="F22" s="19" t="n">
+        <f aca="false">IF(E22,0,C22)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B23" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="C23" s="17" t="n">
+        <v>0.009</v>
+      </c>
+      <c r="D23" s="18" t="b">
+        <v>0</v>
+      </c>
+      <c r="E23" s="19" t="n">
+        <f aca="false">IF(D23,C23,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F23" s="19" t="n">
+        <f aca="false">IF(E23,0,C23)</f>
+        <v>0.009</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C26" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="E26" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="F26" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="G26" s="15" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B27" s="0" t="s">
+        <v>60</v>
+      </c>
+      <c r="C27" s="19" t="n">
+        <f aca="false">SUM(C14:C23)</f>
+        <v>0.643</v>
+      </c>
+      <c r="E27" s="20" t="n">
+        <f aca="false">SUM(E14:E23)</f>
+        <v>0.565</v>
+      </c>
+      <c r="F27" s="19" t="n">
+        <f aca="false">SUM(F14:F23)</f>
+        <v>0.078</v>
+      </c>
+      <c r="G27" s="19" t="n">
+        <f aca="false">1-E27-F27</f>
+        <v>0.357</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C33" s="19"/>
+    </row>
+    <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C34" s="19"/>
+    </row>
+    <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C35" s="19"/>
+    </row>
+    <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C36" s="19"/>
+    </row>
+    <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C37" s="19"/>
+    </row>
+    <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C38" s="19"/>
+    </row>
+    <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C39" s="19"/>
+    </row>
+    <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C40" s="19"/>
+    </row>
+    <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C41" s="19"/>
+    </row>
+    <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C42" s="19"/>
+    </row>
+    <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C43" s="19"/>
+    </row>
+    <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C44" s="19"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A11:C11"/>
+  </mergeCells>
+  <conditionalFormatting sqref="E27">
+    <cfRule type="cellIs" priority="2" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>0.6</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>0.8</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="greaterThanOrEqual" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
+      <formula>0.8</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>